<commit_message>
Add new test cases for washer dryer pedestals
Co-authored-by: nikhil.giri <nikhil.giri@programming.com>
</commit_message>
<xml_diff>
--- a/results/result_11-06-2025_03:38.xlsx
+++ b/results/result_11-06-2025_03:38.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5513" uniqueCount="2450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5541" uniqueCount="2462">
   <si>
     <t>Test ID</t>
   </si>
@@ -7361,6 +7361,42 @@
   </si>
   <si>
     <t>washer and dryer with pedestals (Washer Dryer)</t>
+  </si>
+  <si>
+    <t>TST_787</t>
+  </si>
+  <si>
+    <t>2025-11-06T04:52:34.644Z</t>
+  </si>
+  <si>
+    <t>washer dryer pedestals (Washer Dryer)</t>
+  </si>
+  <si>
+    <t>TST_788</t>
+  </si>
+  <si>
+    <t>2025-11-06T05:07:45.299Z</t>
+  </si>
+  <si>
+    <t>pedestals for washer and dryer (Washer Dryer)</t>
+  </si>
+  <si>
+    <t>TST_789</t>
+  </si>
+  <si>
+    <t>2025-11-06T05:07:53.043Z</t>
+  </si>
+  <si>
+    <t>samsung washer dryer pedestal (Washer Dryer)</t>
+  </si>
+  <si>
+    <t>TST_790</t>
+  </si>
+  <si>
+    <t>2025-11-06T05:08:01.183Z</t>
+  </si>
+  <si>
+    <t>washer pedestal (Washer Dryer)</t>
   </si>
 </sst>
 </file>
@@ -7767,7 +7803,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K787"/>
+  <dimension ref="A1:K791"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -35237,6 +35273,146 @@
         <v>1.01</v>
       </c>
     </row>
+    <row r="788" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A788" t="s">
+        <v>2450</v>
+      </c>
+      <c r="B788" t="s">
+        <v>2451</v>
+      </c>
+      <c r="C788" t="s">
+        <v>13</v>
+      </c>
+      <c r="D788" t="s">
+        <v>2452</v>
+      </c>
+      <c r="E788" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F788" s="1">
+        <v>100</v>
+      </c>
+      <c r="G788" t="s">
+        <v>21</v>
+      </c>
+      <c r="H788">
+        <v>879</v>
+      </c>
+      <c r="I788">
+        <v>200</v>
+      </c>
+      <c r="J788" t="s">
+        <v>17</v>
+      </c>
+      <c r="K788">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="789" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A789" t="s">
+        <v>2453</v>
+      </c>
+      <c r="B789" t="s">
+        <v>2454</v>
+      </c>
+      <c r="C789" t="s">
+        <v>13</v>
+      </c>
+      <c r="D789" t="s">
+        <v>2455</v>
+      </c>
+      <c r="E789" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F789" s="1">
+        <v>100</v>
+      </c>
+      <c r="G789" t="s">
+        <v>21</v>
+      </c>
+      <c r="H789">
+        <v>1446</v>
+      </c>
+      <c r="I789">
+        <v>200</v>
+      </c>
+      <c r="J789" t="s">
+        <v>17</v>
+      </c>
+      <c r="K789">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="790" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A790" t="s">
+        <v>2456</v>
+      </c>
+      <c r="B790" t="s">
+        <v>2457</v>
+      </c>
+      <c r="C790" t="s">
+        <v>13</v>
+      </c>
+      <c r="D790" t="s">
+        <v>2458</v>
+      </c>
+      <c r="E790" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F790" s="1">
+        <v>100</v>
+      </c>
+      <c r="G790" t="s">
+        <v>21</v>
+      </c>
+      <c r="H790">
+        <v>927</v>
+      </c>
+      <c r="I790">
+        <v>200</v>
+      </c>
+      <c r="J790" t="s">
+        <v>17</v>
+      </c>
+      <c r="K790">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="791" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A791" t="s">
+        <v>2459</v>
+      </c>
+      <c r="B791" t="s">
+        <v>2460</v>
+      </c>
+      <c r="C791" t="s">
+        <v>13</v>
+      </c>
+      <c r="D791" t="s">
+        <v>2461</v>
+      </c>
+      <c r="E791" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F791" s="1">
+        <v>100</v>
+      </c>
+      <c r="G791" t="s">
+        <v>21</v>
+      </c>
+      <c r="H791">
+        <v>1199</v>
+      </c>
+      <c r="I791">
+        <v>200</v>
+      </c>
+      <c r="J791" t="s">
+        <v>17</v>
+      </c>
+      <c r="K791">
+        <v>1.22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>